<commit_message>
OPTV-29 complete import task & task-event
</commit_message>
<xml_diff>
--- a/src/styles/task/Task Template.xlsx
+++ b/src/styles/task/Task Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="7510" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
@@ -1116,6 +1116,9 @@
   <sheetPr/>
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelRow="3"/>
+  <cols>
+    <col min="1" max="1" width="136.166666666667" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">

</xml_diff>